<commit_message>
Refine third-bimester workbook after audit
Extend the existing conceptual conditional-formatting rules to the third-bimester column and update Control help text to describe 3B validation and cumulative use of prior-period sources.

Keep the Apps Script unchanged; this addresses the workbook presentation and guidance findings from the independent audit before functional fixture validation.
</commit_message>
<xml_diff>
--- a/src/Generador_informes_individuales_EPS_v0_3.xlsx
+++ b/src/Generador_informes_individuales_EPS_v0_3.xlsx
@@ -14926,6 +14926,17 @@
       <x:formula>"Avanzado"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G9:G16">
+    <x:cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+      <x:formula>"En Proceso"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="1" priority="5" operator="equal">
+      <x:formula>"Suficiente"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="0" priority="6" operator="equal">
+      <x:formula>"Avanzado"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree1e090b917046da"/>
 </x:worksheet>
@@ -15127,7 +15138,7 @@
       <x:c r="C16" s="102" t="str"/>
       <x:c r="D16" s="102" t="str"/>
       <x:c r="E16" s="102" t="str">
-        <x:v>1º bimestre</x:v>
+        <x:v>1º y 3º bimestre</x:v>
       </x:c>
       <x:c r="F16" s="102" t="str">
         <x:v>En proceso; Suficiente; Avanzado; ACREDITÓ</x:v>
@@ -15215,7 +15226,7 @@
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
       <x:c r="A24" s="99" t="str">
-        <x:v>El boletín de 1º cuatrimestre es acumulativo: incluye materias con valoración válida en 1º bimestre y/o 1º cuatrimestre.</x:v>
+        <x:v>Los informes de 1º cuatrimestre y 3º bimestre son acumulativos respecto de períodos anteriores. Para generar el 3º bimestre, pueden usarse fuentes de 1º bimestre y 1º cuatrimestre como antecedentes.</x:v>
       </x:c>
       <x:c r="B24" s="99" t="str"/>
       <x:c r="C24" s="99" t="str"/>

</xml_diff>

<commit_message>
Agregar generación de boletines por curso
Generar un libro nuevo con una hoja por estudiante listo para exportar, reutilizar la lógica del informe individual, mantener las fuentes de sólo lectura y agregar el selector de nivel y el resumen oculto de la tanda.
</commit_message>
<xml_diff>
--- a/src/Generador_informes_individuales_EPS_v0_3.xlsx
+++ b/src/Generador_informes_individuales_EPS_v0_3.xlsx
@@ -15059,9 +15059,13 @@
       <x:c r="F8" s="102" t="str"/>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
-      <x:c r="A9" s="90" t="str"/>
+      <x:c r="A9" s="90" t="str">
+        <x:v>Nivel / curso</x:v>
+      </x:c>
       <x:c r="B9" s="102" t="str"/>
-      <x:c r="C9" s="102" t="str"/>
+      <x:c r="C9" s="102" t="str">
+        <x:v>Sólo para la generación por curso. Valores posibles: EPS1, EPS2, EPS3 o EPS4. La generación individual lo ignora.</x:v>
+      </x:c>
       <x:c r="D9" s="102" t="str"/>
       <x:c r="E9" s="102" t="str"/>
       <x:c r="F9" s="102" t="str"/>
@@ -15255,12 +15259,15 @@
       <x:c r="F26" s="99" t="str"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B5">
       <x:formula1>"1º bimestre,1º cuatrimestre,3º bimestre"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="B6">
       <x:formula1>"EPSI,EPSG"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="B9">
+      <x:formula1>"EPS1,EPS2,EPS3,EPS4"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Compactar Control y aclarar el contrato de la fuente principal
Elimina la fila vacía de Control y alinea las fuentes en B10, B11 y B12. Aclara que LISTO PARA EXPORTAR se exige sólo en la fuente principal y refuerza ese contrato y las coordenadas reales con pruebas.
</commit_message>
<xml_diff>
--- a/src/Generador_informes_individuales_EPS_v0_3.xlsx
+++ b/src/Generador_informes_individuales_EPS_v0_3.xlsx
@@ -15083,144 +15083,146 @@
       <x:c r="F10" s="102" t="str"/>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
-      <x:c r="A11" s="90" t="str"/>
+      <x:c r="A11" s="90" t="str">
+        <x:v>URL o ID del archivo de valoraciones del 1º cuatrimestre</x:v>
+      </x:c>
       <x:c r="B11" s="102" t="str"/>
-      <x:c r="C11" s="102" t="str"/>
+      <x:c r="C11" s="102" t="str">
+        <x:v>Fuente principal cuando se genera 1º cuatrimestre.</x:v>
+      </x:c>
       <x:c r="D11" s="102" t="str"/>
       <x:c r="E11" s="102" t="str"/>
       <x:c r="F11" s="102" t="str"/>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
       <x:c r="A12" s="90" t="str">
-        <x:v>URL o ID del archivo de valoraciones del 1º cuatrimestre</x:v>
+        <x:v>URL o ID del archivo de valoraciones del 3º bimestre</x:v>
       </x:c>
       <x:c r="B12" s="102" t="str"/>
       <x:c r="C12" s="102" t="str">
-        <x:v>Fuente principal cuando se genera 1º cuatrimestre.</x:v>
+        <x:v>Fuente del 3º bimestre.</x:v>
       </x:c>
       <x:c r="D12" s="102" t="str"/>
       <x:c r="E12" s="102" t="str"/>
       <x:c r="F12" s="102" t="str"/>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
-      <x:c r="A13" s="90" t="str">
-        <x:v>URL o ID del archivo de valoraciones del 3º bimestre</x:v>
-      </x:c>
+      <x:c r="A13" s="102" t="str"/>
       <x:c r="B13" s="102" t="str"/>
-      <x:c r="C13" s="102" t="str">
-        <x:v>Fuente del 3º bimestre.</x:v>
-      </x:c>
+      <x:c r="C13" s="102" t="str"/>
       <x:c r="D13" s="102" t="str"/>
       <x:c r="E13" s="102" t="str"/>
       <x:c r="F13" s="102" t="str"/>
     </x:row>
-    <x:row r="14" ht="22" customHeight="1">
-      <x:c r="A14" s="102" t="str"/>
-      <x:c r="B14" s="102" t="str"/>
-      <x:c r="C14" s="102" t="str"/>
-      <x:c r="D14" s="102" t="str"/>
-      <x:c r="E14" s="102" t="str"/>
-      <x:c r="F14" s="102" t="str"/>
-    </x:row>
-    <x:row r="15" ht="30" customHeight="1">
-      <x:c r="A15" s="82" t="str">
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="82" t="str">
         <x:v>Manual breve</x:v>
       </x:c>
-      <x:c r="B15" s="82" t="str"/>
-      <x:c r="C15" s="82" t="str"/>
-      <x:c r="D15" s="102" t="str"/>
-      <x:c r="E15" s="82" t="str">
+      <x:c r="B14" s="82" t="str"/>
+      <x:c r="C14" s="82" t="str"/>
+      <x:c r="D14" s="102" t="str"/>
+      <x:c r="E14" s="82" t="str">
         <x:v>Valores válidos</x:v>
       </x:c>
-      <x:c r="F15" s="82" t="str"/>
+      <x:c r="F14" s="82" t="str"/>
+    </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" s="102" t="str">
+        <x:v>1. Elegir período: 1º bimestre, 1º cuatrimestre o 3º bimestre.</x:v>
+      </x:c>
+      <x:c r="B15" s="102" t="str"/>
+      <x:c r="C15" s="102" t="str"/>
+      <x:c r="D15" s="102" t="str"/>
+      <x:c r="E15" s="102" t="str">
+        <x:v>1º y 3º bimestre</x:v>
+      </x:c>
+      <x:c r="F15" s="102" t="str">
+        <x:v>En proceso; Suficiente; Avanzado; ACREDITÓ</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="102" t="str">
-        <x:v>1. Elegir período: 1º bimestre, 1º cuatrimestre o 3º bimestre.</x:v>
+        <x:v>2. Elegir hoja origen: EPSI o EPSG.</x:v>
       </x:c>
       <x:c r="B16" s="102" t="str"/>
       <x:c r="C16" s="102" t="str"/>
       <x:c r="D16" s="102" t="str"/>
       <x:c r="E16" s="102" t="str">
-        <x:v>1º y 3º bimestre</x:v>
+        <x:v>1º cuatrimestre</x:v>
       </x:c>
       <x:c r="F16" s="102" t="str">
-        <x:v>En proceso; Suficiente; Avanzado; ACREDITÓ</x:v>
+        <x:v>Enteros 1 a 10; ACREDITÓ</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="102" t="str">
-        <x:v>2. Elegir hoja origen: EPSI o EPSG.</x:v>
+        <x:v>3. Ingresar DNI y verificar las URL/ID de fuentes.</x:v>
       </x:c>
       <x:c r="B17" s="102" t="str"/>
       <x:c r="C17" s="102" t="str"/>
       <x:c r="D17" s="102" t="str"/>
       <x:c r="E17" s="102" t="str">
-        <x:v>1º cuatrimestre</x:v>
+        <x:v>Excluidos</x:v>
       </x:c>
       <x:c r="F17" s="102" t="str">
-        <x:v>Enteros 1 a 10; ACREDITÓ</x:v>
+        <x:v>vacío; NO CURSA; CURSA</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="A18" s="102" t="str">
-        <x:v>3. Ingresar DNI y verificar las URL/ID de fuentes.</x:v>
+        <x:v>4. Ejecutar Informes EPS &gt; Generar informe actual.</x:v>
       </x:c>
       <x:c r="B18" s="102" t="str"/>
       <x:c r="C18" s="102" t="str"/>
       <x:c r="D18" s="102" t="str"/>
       <x:c r="E18" s="102" t="str">
-        <x:v>Excluidos</x:v>
+        <x:v>No válidos 1º cuat.</x:v>
       </x:c>
       <x:c r="F18" s="102" t="str">
-        <x:v>vacío; NO CURSA; CURSA</x:v>
+        <x:v>decimales; texto junto con número; nota escrita como texto</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19" s="102" t="str">
-        <x:v>4. Ejecutar Informes EPS &gt; Generar informe actual.</x:v>
+        <x:v>5. Revisar Informe_actual antes de imprimir o exportar.</x:v>
       </x:c>
       <x:c r="B19" s="102" t="str"/>
       <x:c r="C19" s="102" t="str"/>
       <x:c r="D19" s="102" t="str"/>
-      <x:c r="E19" s="102" t="str">
-        <x:v>No válidos 1º cuat.</x:v>
-      </x:c>
-      <x:c r="F19" s="102" t="str">
-        <x:v>decimales; texto junto con número; nota escrita como texto</x:v>
-      </x:c>
+      <x:c r="E19" s="102" t="str"/>
+      <x:c r="F19" s="102" t="str"/>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
-      <x:c r="A20" s="102" t="str">
-        <x:v>5. Revisar Informe_actual antes de imprimir o exportar.</x:v>
-      </x:c>
+      <x:c r="A20" s="102" t="str"/>
       <x:c r="B20" s="102" t="str"/>
       <x:c r="C20" s="102" t="str"/>
       <x:c r="D20" s="102" t="str"/>
       <x:c r="E20" s="102" t="str"/>
       <x:c r="F20" s="102" t="str"/>
     </x:row>
-    <x:row r="21" ht="22" customHeight="1">
-      <x:c r="A21" s="102" t="str"/>
-      <x:c r="B21" s="102" t="str"/>
-      <x:c r="C21" s="102" t="str"/>
-      <x:c r="D21" s="102" t="str"/>
-      <x:c r="E21" s="102" t="str"/>
-      <x:c r="F21" s="102" t="str"/>
-    </x:row>
-    <x:row r="22" ht="30" customHeight="1">
-      <x:c r="A22" s="82" t="str">
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="82" t="str">
         <x:v>Reglas centrales</x:v>
       </x:c>
-      <x:c r="B22" s="82" t="str"/>
-      <x:c r="C22" s="82" t="str"/>
-      <x:c r="D22" s="82" t="str"/>
-      <x:c r="E22" s="82" t="str"/>
-      <x:c r="F22" s="82" t="str"/>
+      <x:c r="B21" s="82" t="str"/>
+      <x:c r="C21" s="82" t="str"/>
+      <x:c r="D21" s="82" t="str"/>
+      <x:c r="E21" s="82" t="str"/>
+      <x:c r="F21" s="82" t="str"/>
+    </x:row>
+    <x:row r="22" ht="30" customHeight="1">
+      <x:c r="A22" s="99" t="str">
+        <x:v>La hoja origen es única y representa la orientación: EPSI o EPSG.</x:v>
+      </x:c>
+      <x:c r="B22" s="99" t="str"/>
+      <x:c r="C22" s="99" t="str"/>
+      <x:c r="D22" s="99" t="str"/>
+      <x:c r="E22" s="99" t="str"/>
+      <x:c r="F22" s="99" t="str"/>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
       <x:c r="A23" s="99" t="str">
-        <x:v>La hoja origen es única y representa la orientación: EPSI o EPSG.</x:v>
+        <x:v>Los informes de 1º cuatrimestre y 3º bimestre son acumulativos respecto de períodos anteriores. Para generar el 3º bimestre, pueden usarse fuentes de 1º bimestre y 1º cuatrimestre como antecedentes.</x:v>
       </x:c>
       <x:c r="B23" s="99" t="str"/>
       <x:c r="C23" s="99" t="str"/>
@@ -15230,7 +15232,7 @@
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
       <x:c r="A24" s="99" t="str">
-        <x:v>Los informes de 1º cuatrimestre y 3º bimestre son acumulativos respecto de períodos anteriores. Para generar el 3º bimestre, pueden usarse fuentes de 1º bimestre y 1º cuatrimestre como antecedentes.</x:v>
+        <x:v>Las celdas de períodos sin calificación válida quedan vacías; no se completan con guion.</x:v>
       </x:c>
       <x:c r="B24" s="99" t="str"/>
       <x:c r="C24" s="99" t="str"/>
@@ -15240,23 +15242,13 @@
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
       <x:c r="A25" s="99" t="str">
-        <x:v>Las celdas de períodos sin calificación válida quedan vacías; no se completan con guion.</x:v>
+        <x:v>La información general sale siempre de la fuente principal del período generado.</x:v>
       </x:c>
       <x:c r="B25" s="99" t="str"/>
       <x:c r="C25" s="99" t="str"/>
       <x:c r="D25" s="99" t="str"/>
       <x:c r="E25" s="99" t="str"/>
       <x:c r="F25" s="99" t="str"/>
-    </x:row>
-    <x:row r="26" ht="30" customHeight="1">
-      <x:c r="A26" s="99" t="str">
-        <x:v>La información general sale siempre de la fuente principal del período generado.</x:v>
-      </x:c>
-      <x:c r="B26" s="99" t="str"/>
-      <x:c r="C26" s="99" t="str"/>
-      <x:c r="D26" s="99" t="str"/>
-      <x:c r="E26" s="99" t="str"/>
-      <x:c r="F26" s="99" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="3">

</xml_diff>